<commit_message>
feat(api): update demo user configurations and enhance advice functionality
- Updated .env.example and docker-compose.yml to reflect changes in demo user emails and roles for improved clarity.
- Enhanced README.md to provide updated login credentials for demo users, aligning with the new configurations.
- Introduced advice functionality in the remarks service, allowing developers to provide suggestions on remarks awaiting PM review.
- Updated remarks controller to handle advice submissions and retractions, ensuring real-time updates for PM visibility.
- Improved data models to include advice details, enhancing the context for remarks and facilitating better decision-making.

This commit significantly improves the demo experience and enhances the collaborative workflow between developers and PMs through the new advice feature.
</commit_message>
<xml_diff>
--- a/apps/web/public/template.xlsx
+++ b/apps/web/public/template.xlsx
@@ -47,7 +47,7 @@
     <comment ref="E1" authorId="0">
       <text>
         <r>
-          <t>low / medium / high — необязательно</t>
+          <t>высокая / средняя / низкая — необязательно</t>
         </r>
       </text>
     </comment>
@@ -65,22 +65,22 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
-    <t>external_id</t>
+    <t>№</t>
   </si>
   <si>
-    <t>page_or_screen</t>
+    <t>Где</t>
   </si>
   <si>
-    <t>description</t>
+    <t>Что не так</t>
   </si>
   <si>
-    <t>expected</t>
+    <t>Как должно быть</t>
   </si>
   <si>
-    <t>severity</t>
+    <t>Важность</t>
   </si>
   <si>
-    <t>screenshot</t>
+    <t>Скрин</t>
   </si>
 </sst>
 </file>

</xml_diff>